<commit_message>
Added  Checks and clearing schedule
</commit_message>
<xml_diff>
--- a/Project/PlanningCenterScheduleUploader/PlanningCenterAPI.Test/Schedule.xlsx
+++ b/Project/PlanningCenterScheduleUploader/PlanningCenterAPI.Test/Schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\GitHub\PlanningCenterScheduleUploader\Project\PlanningCenterScheduleUploader\PlanningCenterAPI.Test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7374EE1-0DA1-4EBC-BC96-867D96C254CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3652E56A-1880-4102-9561-E87448340688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{270EC0F9-CA9F-4B8F-8137-AAC43B2367E2}"/>
   </bookViews>
@@ -40,40 +40,40 @@
     <t>Service Type</t>
   </si>
   <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>Camera</t>
+  </si>
+  <si>
+    <t>Editor</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Ransome Madziwa</t>
+  </si>
+  <si>
+    <t>Ramon Ferreira</t>
+  </si>
+  <si>
+    <t>Wale Adeniran</t>
+  </si>
+  <si>
+    <t>Devlyn van der Walt</t>
+  </si>
+  <si>
+    <t>Connor Milne</t>
+  </si>
+  <si>
     <t>Sunday and Other Services</t>
   </si>
   <si>
-    <t>Team</t>
-  </si>
-  <si>
     <t>Live Stream</t>
   </si>
   <si>
-    <t>Camera</t>
-  </si>
-  <si>
     <t>Comms</t>
-  </si>
-  <si>
-    <t>Editor</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Ransome Madziwa</t>
-  </si>
-  <si>
-    <t>Ramon Ferreira</t>
-  </si>
-  <si>
-    <t>Wale Adeniran</t>
-  </si>
-  <si>
-    <t>Devlyn van der Walt</t>
-  </si>
-  <si>
-    <t>Connor Milne</t>
   </si>
 </sst>
 </file>
@@ -449,16 +449,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -466,13 +466,13 @@
         <v>46115</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -480,13 +480,13 @@
         <v>46117</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -494,13 +494,13 @@
         <v>46124</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D4" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -508,13 +508,13 @@
         <v>46131</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D5" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -522,13 +522,13 @@
         <v>46138</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D6" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -551,15 +551,15 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
New pipeline validation is in place now
</commit_message>
<xml_diff>
--- a/Project/PlanningCenterScheduleUploader/PlanningCenterAPI.Test/Schedule.xlsx
+++ b/Project/PlanningCenterScheduleUploader/PlanningCenterAPI.Test/Schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\GitHub\PlanningCenterScheduleUploader\Project\PlanningCenterScheduleUploader\PlanningCenterAPI.Test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3652E56A-1880-4102-9561-E87448340688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E52A05EF-F2A4-4C41-BF00-83DAC23F62DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{270EC0F9-CA9F-4B8F-8137-AAC43B2367E2}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="15">
   <si>
     <t>Service Type</t>
   </si>
@@ -43,9 +43,6 @@
     <t>Team</t>
   </si>
   <si>
-    <t>Camera</t>
-  </si>
-  <si>
     <t>Editor</t>
   </si>
   <si>
@@ -55,9 +52,6 @@
     <t>Ransome Madziwa</t>
   </si>
   <si>
-    <t>Ramon Ferreira</t>
-  </si>
-  <si>
     <t>Wale Adeniran</t>
   </si>
   <si>
@@ -74,6 +68,18 @@
   </si>
   <si>
     <t>Comms</t>
+  </si>
+  <si>
+    <t>Camera First Service</t>
+  </si>
+  <si>
+    <t>Camera Second Service</t>
+  </si>
+  <si>
+    <t>Byron Raaff</t>
+  </si>
+  <si>
+    <t>Tando Khoza</t>
   </si>
 </sst>
 </file>
@@ -439,96 +445,115 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDCAD8E2-0228-42F9-9D20-C4D47ACFB5CC}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="19" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>12</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>46115</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>46117</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+      <c r="E3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>46124</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>46131</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="E5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>46138</v>
       </c>
       <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" t="s">
         <v>6</v>
       </c>
-      <c r="C6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D6" t="s">
-        <v>8</v>
+      <c r="E6" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -551,7 +576,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -559,7 +584,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>